<commit_message>
sharpe annuality to daily
</commit_message>
<xml_diff>
--- a/fixed_allocation_daily_volatile.xlsx
+++ b/fixed_allocation_daily_volatile.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:M45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2229,6 +2229,516 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2025-09-13T10:52:58</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>trial_001</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>0.1513</v>
+      </c>
+      <c r="F36" t="n">
+        <v>1.3594</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0.1669</v>
+      </c>
+      <c r="H36" t="n">
+        <v>-0.0898</v>
+      </c>
+      <c r="I36" t="n">
+        <v>0.1187</v>
+      </c>
+      <c r="J36" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K36" t="n">
+        <v>-0.1017</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 313}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2025-09-13T10:58:10</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>trial_002</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>0.1178</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1.1137</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0.1298</v>
+      </c>
+      <c r="H37" t="n">
+        <v>-0.1163</v>
+      </c>
+      <c r="I37" t="n">
+        <v>0.1156</v>
+      </c>
+      <c r="J37" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K37" t="n">
+        <v>-0.0747</v>
+      </c>
+      <c r="L37" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 314}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2025-09-13T11:03:19</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>trial_003</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E38" t="n">
+        <v>0.1859</v>
+      </c>
+      <c r="F38" t="n">
+        <v>1.612</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0.2054</v>
+      </c>
+      <c r="H38" t="n">
+        <v>-0.0624</v>
+      </c>
+      <c r="I38" t="n">
+        <v>0.1204</v>
+      </c>
+      <c r="J38" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K38" t="n">
+        <v>-0.1032</v>
+      </c>
+      <c r="L38" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 315}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2025-09-13T11:08:20</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>trial_004</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>0.1638</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1.3964</v>
+      </c>
+      <c r="G39" t="n">
+        <v>0.1808</v>
+      </c>
+      <c r="H39" t="n">
+        <v>-0.0799</v>
+      </c>
+      <c r="I39" t="n">
+        <v>0.1246</v>
+      </c>
+      <c r="J39" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K39" t="n">
+        <v>-0.0829</v>
+      </c>
+      <c r="L39" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 316}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2025-09-13T11:13:25</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>trial_005</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>0.163</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.414</v>
+      </c>
+      <c r="G40" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-0.0805</v>
+      </c>
+      <c r="I40" t="n">
+        <v>0.1223</v>
+      </c>
+      <c r="J40" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K40" t="n">
+        <v>-0.1031</v>
+      </c>
+      <c r="L40" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 317}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-09-13T11:18:34</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>trial_006</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>0.1729</v>
+      </c>
+      <c r="F41" t="n">
+        <v>1.4545</v>
+      </c>
+      <c r="G41" t="n">
+        <v>0.1909</v>
+      </c>
+      <c r="H41" t="n">
+        <v>-0.0728</v>
+      </c>
+      <c r="I41" t="n">
+        <v>0.1255</v>
+      </c>
+      <c r="J41" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K41" t="n">
+        <v>-0.1028</v>
+      </c>
+      <c r="L41" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 318}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-09-13T11:23:53</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>trial_007</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E42" t="n">
+        <v>0.2121</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.8237</v>
+      </c>
+      <c r="G42" t="n">
+        <v>0.2346</v>
+      </c>
+      <c r="H42" t="n">
+        <v>-0.0417</v>
+      </c>
+      <c r="I42" t="n">
+        <v>0.1195</v>
+      </c>
+      <c r="J42" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K42" t="n">
+        <v>-0.0849</v>
+      </c>
+      <c r="L42" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 319}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-09-13T11:28:48</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>trial_008</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>0.1829</v>
+      </c>
+      <c r="F43" t="n">
+        <v>1.6189</v>
+      </c>
+      <c r="G43" t="n">
+        <v>0.2021</v>
+      </c>
+      <c r="H43" t="n">
+        <v>-0.0648</v>
+      </c>
+      <c r="I43" t="n">
+        <v>0.118</v>
+      </c>
+      <c r="J43" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K43" t="n">
+        <v>-0.0895</v>
+      </c>
+      <c r="L43" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 320}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-09-13T11:33:53</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>trial_009</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>0.1326</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1.2426</v>
+      </c>
+      <c r="G44" t="n">
+        <v>0.1462</v>
+      </c>
+      <c r="H44" t="n">
+        <v>-0.1046</v>
+      </c>
+      <c r="I44" t="n">
+        <v>0.1151</v>
+      </c>
+      <c r="J44" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K44" t="n">
+        <v>-0.079</v>
+      </c>
+      <c r="L44" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 321}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-09-13T11:39:04</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>FIXED_td3_allocation_daily_volatile_runs_batch</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>trial_010</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>td3</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>0.1417</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.3491</v>
+      </c>
+      <c r="G45" t="n">
+        <v>0.1562</v>
+      </c>
+      <c r="H45" t="n">
+        <v>-0.0974</v>
+      </c>
+      <c r="I45" t="n">
+        <v>0.1123</v>
+      </c>
+      <c r="J45" t="n">
+        <v>0.1233</v>
+      </c>
+      <c r="K45" t="n">
+        <v>-0.0873</v>
+      </c>
+      <c r="L45" t="n">
+        <v>-0.0897</v>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>{"erl": {"learning_rate": 1.3204392685000274e-05, "batch_size": 512, "gamma": 0.9954379276836015, "net_dimension": 256, "net_dims": [256, 256], "target_step": 8192, "horizon_len": 2048, "repeat_times": 2.0, "buffer_size": 1000000, "buffer_init_size": 2048, "eval_gap": 64, "eval_times": 16, "if_use_per": false, "seed": 322}, "task": "allocation", "freq": "daily", "dataset": "volatile"}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>